<commit_message>
GSB 5ba340b1-4d62-513e-aa7c-90cf93aaa93c A: platform archive
</commit_message>
<xml_diff>
--- a/samples/sample_impact.xlsx
+++ b/samples/sample_impact.xlsx
@@ -13,9 +13,18 @@
     <sheet name="月报 2026" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="循环" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="数据" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="审计示例" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="名称" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="审计示例" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="税率">参数!$B$5</definedName>
+    <definedName name="参数表_单价区">参数!$B$2:$B$3</definedName>
+    <definedName name="常量_PI">3.14</definedName>
+    <definedName name="坏名_引用错误">#REF!</definedName>
+    <definedName name="坏名_幽灵表">不存在的表!$A$1</definedName>
+    <definedName name="折扣" localSheetId="0">参数!$B$4</definedName>
+    <definedName name="折扣" localSheetId="6">名称!$A$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -2392,6 +2401,125 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>场景</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>公式</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>工作簿级税率</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>税率*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>本表工作表级折扣</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>折扣*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>限定参数表同名折扣</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>参数!折扣*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>区域名称求和</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>SUM(参数表_单价区)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>常量名称</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>常量_PI*2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>损坏名称(#REF!)</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>坏名_引用错误+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>名称指向缺失工作表</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>坏名_幽灵表+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>未定义名称</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>从未定义的名称+1</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
GSB 5ba340b1-4d62-513e-aa7c-90cf93aaa93c B: platform archive
</commit_message>
<xml_diff>
--- a/samples/sample_impact.xlsx
+++ b/samples/sample_impact.xlsx
@@ -14,8 +14,26 @@
     <sheet name="循环" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="数据" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="审计示例" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="名称" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="单价">参数!$B$2</definedName>
+    <definedName name="数量">参数!$B$3</definedName>
+    <definedName name="折扣">参数!$B$2</definedName>
+    <definedName name="数据列">数据!$B$2:$B$201</definedName>
+    <definedName name="月数">参数!$B$6</definedName>
+    <definedName name="年化系数">月数</definedName>
+    <definedName name="折后小计">参数!$B$2*参数!$B$3*参数!$B$4</definedName>
+    <definedName name="税率常量">0.13</definedName>
+    <definedName name="失效名称">#REF!</definedName>
+    <definedName name="幽灵表名称">不存在的表!$A$1</definedName>
+    <definedName name="外部预算">[1]年度预算.xlsx!汇总!$B$2</definedName>
+    <definedName name="越界数据名">数据!$B$999</definedName>
+    <definedName name="环甲">环乙</definedName>
+    <definedName name="环乙">环甲</definedName>
+    <definedName name="系数" localSheetId="1">参数!$B$4</definedName>
+    <definedName name="折扣" localSheetId="7">参数!$B$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -2475,4 +2493,194 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>单价（工作簿级名称 单价 → 参数!B2）</t>
+        </is>
+      </c>
+      <c r="B1">
+        <f>单价</f>
+        <v/>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>数量（工作簿级名称 数量 → 参数!B3）</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>单价*数量</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>折扣金额（工作表级名称 折扣 → 参数!B4，遮蔽全局）</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>折扣</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>跨表引用计算表本地名称（计算!系数）</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>计算!系数</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>区域名称（数据列 → 数据!B2:B201）</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>SUM(数据列)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>嵌套名称（年化系数 → 月数 → 参数!B6）</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>年化系数</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>公式表达式名称（折后小计 = 单价*数量*折扣率）</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>折后小计</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>常量名称（税率常量 0.13，不产生依赖边）</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>税率常量</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>未定义名称（error: undefined_name）</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>不存在的名称+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>已删除引用名称（error: invalid_name，#REF!）</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>失效名称</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>指向不存在工作表的名称（error: missing_sheet）</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>幽灵表名称</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>限定到不存在工作表的名称（error: undefined_name）</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>不存在的表!某名称</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>外部工作簿名称（warning: external_name）</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>外部预算</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>经名称越界引用（warning: out_of_range）</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>越界数据名</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>名称循环（环甲→环乙→环甲，error: invalid_name）</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>环甲</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>名称链下游（验证影响面经名称传播）</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>B2*年化系数</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>